<commit_message>
docs: extend WBS with Master + Excel Upload modules (50 checks, 119.5h total)
Live-discovered from the ERP sidebar and added to WBS_CRM_TaskManagement.xlsx:
- Master (22.5h / 10 checks): Business Contacts, Users, Reset Password, Branch,
  User Role Groups (permission matrix), Teams, Client Settings, Custom Fields,
  Dynamic Reports builder, Field Mapping.
- Excel Upload (13h / 5 checks): Individual/Business Customer, Enquiry, Project,
  Solar Project uploads — each with template/valid/invalid/duplicate/verify matrix.
Dashboard now summarizes 4 modules. Totals: CRM 45.5h + TM 38.5h + Master 22.5h
+ Excel Upload 13h = 119.5h across 50 page-wise checks.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel/WBS_CRM_TaskManagement.xlsx
+++ b/docs/excel/WBS_CRM_TaskManagement.xlsx
@@ -181,8 +181,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WBS" displayName="WBS" ref="A1:L36" headerRowCount="1">
-  <autoFilter ref="A1:L36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WBS" displayName="WBS" ref="A1:L51" headerRowCount="1">
+  <autoFilter ref="A1:L51"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Project"/>
     <tableColumn id="2" name="Module"/>
@@ -505,8 +505,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:L52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -2230,23 +2230,728 @@
       <c r="L36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="F37" s="4" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Progbiz ERP</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Business Contacts</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Business contacts master (/business-contacts)</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>List, create, edit, search, duplicate handling</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Standard CRUD master + search modes</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H37" s="3" t="n"/>
+      <c r="I37" s="2" t="n"/>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K37" s="3">
+        <f>G37-H37</f>
+        <v/>
+      </c>
+      <c r="L37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Progbiz ERP</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>User management (/users)</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Create user, assign role, edit, activate/deactivate, login as new user</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>User creation affects auth; verify with a real login</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H38" s="3" t="n"/>
+      <c r="I38" s="2" t="n"/>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K38" s="3">
+        <f>G38-H38</f>
+        <v/>
+      </c>
+      <c r="L38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Progbiz ERP</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Reset password (/change-user-password)</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Change a user's password, old password invalid, new one logs in</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>2-login verification per change</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H39" s="3" t="n"/>
+      <c r="I39" s="2" t="n"/>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K39" s="3">
+        <f>G39-H39</f>
+        <v/>
+      </c>
+      <c r="L39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Progbiz ERP</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Branch master (/branches)</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Create/edit branch, appears in branch dropdowns (task/enquiry forms)</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>CRUD + cross-module dropdown effect</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H40" s="3" t="n"/>
+      <c r="I40" s="2" t="n"/>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K40" s="3">
+        <f>G40-H40</f>
+        <v/>
+      </c>
+      <c r="L40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Progbiz ERP</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>User Role Groups</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Role groups &amp; permissions (/user-role-groups)</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Create group, permission matrix on/off, menu visibility per role</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Permission matrix = many toggle-effect checks with role login</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H41" s="3" t="n"/>
+      <c r="I41" s="2" t="n"/>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K41" s="3">
+        <f>G41-H41</f>
+        <v/>
+      </c>
+      <c r="L41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Progbiz ERP</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Teams master (/teams)</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Create team, add/remove members, team reflected in task/project assignment</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>CRUD + effect check in 2 modules</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H42" s="3" t="n"/>
+      <c r="I42" s="2" t="n"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K42" s="3">
+        <f>G42-H42</f>
+        <v/>
+      </c>
+      <c r="L42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Progbiz ERP</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Client Settings</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Client settings (/client-setting)</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Settings toggles, save, verify each toggle's effect on the app</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Each setting needs an effect verification, not just save</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H43" s="3" t="n"/>
+      <c r="I43" s="2" t="n"/>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K43" s="3">
+        <f>G43-H43</f>
+        <v/>
+      </c>
+      <c r="L43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Progbiz ERP</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Custom Fields</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Custom/dynamic fields (/dynamic-fields)</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Create field per entity, appears on target form, data saves &amp; displays</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Field-type matrix (text/date/select) x target forms</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H44" s="3" t="n"/>
+      <c r="I44" s="2" t="n"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K44" s="3">
+        <f>G44-H44</f>
+        <v/>
+      </c>
+      <c r="L44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Progbiz ERP</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Dynamic Reports</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Dynamic report builder (/dynamic-list)</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Create report (Leads/Tasks/Customers/Project), field picker, filters, generate &amp; verify data</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>4 report types; builder + output correctness</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H45" s="3" t="n"/>
+      <c r="I45" s="2" t="n"/>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K45" s="3">
+        <f>G45-H45</f>
+        <v/>
+      </c>
+      <c r="L45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Progbiz ERP</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Field Mapping</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Field mapping tags (/field-map-tags)</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Create/edit mapping tags, used correctly in templates/reports</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Small master; effect check in one consumer</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H46" s="3" t="n"/>
+      <c r="I46" s="2" t="n"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K46" s="3">
+        <f>G46-H46</f>
+        <v/>
+      </c>
+      <c r="L46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Progbiz ERP</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Excel Upload</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Individual Customer</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Individual customer upload (/individual-customer-upload)</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Template download, valid file upload, invalid/missing-column file, duplicate rows, data verification in Customers</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>5 checks incl. negative files; verify rows landed</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H47" s="3" t="n"/>
+      <c r="I47" s="2" t="n"/>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K47" s="3">
+        <f>G47-H47</f>
+        <v/>
+      </c>
+      <c r="L47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Progbiz ERP</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Excel Upload</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Business Customer</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Business customer upload (/business-customer-upload)</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Same matrix as individual: template, valid, invalid, duplicates, verification</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Mirrors individual-customer flow with business fields</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H48" s="3" t="n"/>
+      <c r="I48" s="2" t="n"/>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K48" s="3">
+        <f>G48-H48</f>
+        <v/>
+      </c>
+      <c r="L48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Progbiz ERP</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Excel Upload</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Enquiry Upload</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Enquiry upload (/enquiry-upload)</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Template, valid upload creates leads, invalid rows report, duplicate phone handling, leads visible in CRM listing</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Creates CRM data — cross-module verification is slower</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H49" s="3" t="n"/>
+      <c r="I49" s="2" t="n"/>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K49" s="3">
+        <f>G49-H49</f>
+        <v/>
+      </c>
+      <c r="L49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Progbiz ERP</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Excel Upload</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Project Upload</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Project upload (/projects-upload)</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Template, valid upload, invalid rows, projects visible in Projects list</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Cross-check in Project module</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H50" s="3" t="n"/>
+      <c r="I50" s="2" t="n"/>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K50" s="3">
+        <f>G50-H50</f>
+        <v/>
+      </c>
+      <c r="L50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Progbiz ERP</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Excel Upload</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Solar Project Upload</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Solar project upload (/solar-project-upload)</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Template, valid upload, invalid rows, solar projects listed</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Variant of project upload with solar fields</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H51" s="3" t="n"/>
+      <c r="I51" s="2" t="n"/>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K51" s="3">
+        <f>G51-H51</f>
+        <v/>
+      </c>
+      <c r="L51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="F52" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="G37" s="5">
-        <f>SUM(G2:G36)</f>
-        <v/>
-      </c>
-      <c r="H37" s="5">
-        <f>SUM(H2:H36)</f>
+      <c r="G52" s="5">
+        <f>SUM(G2:G51)</f>
+        <v/>
+      </c>
+      <c r="H52" s="5">
+        <f>SUM(H2:H51)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pending,In Progress,Completed,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2264,7 +2969,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -2322,7 +3027,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -2337,7 +3042,7 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>WBS DASHBOARD — CRM + Task Management</t>
+          <t>WBS DASHBOARD — CRM · Task Management · Master · Excel Upload</t>
         </is>
       </c>
     </row>
@@ -2461,37 +3166,107 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B7" s="4">
-        <f>SUM(B5:B6)</f>
-        <v/>
-      </c>
-      <c r="C7" s="4">
-        <f>SUM(C5:C6)</f>
-        <v/>
-      </c>
-      <c r="D7" s="4">
-        <f>SUM(D5:D6)</f>
-        <v/>
-      </c>
-      <c r="E7" s="4">
-        <f>SUM(E5:E6)</f>
-        <v/>
-      </c>
-      <c r="F7" s="4">
-        <f>SUM(F5:F6)</f>
-        <v/>
-      </c>
-      <c r="G7" s="4">
-        <f>SUM(G5:G6)</f>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>COUNTIF('WBS Tracker'!B:B,A7)</f>
+        <v/>
+      </c>
+      <c r="C7">
+        <f>COUNTIFS('WBS Tracker'!B:B,A7,'WBS Tracker'!J:J,"Completed")</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>B7-C7</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>SUMIF('WBS Tracker'!B:B,A7,'WBS Tracker'!G:G)</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>SUMIF('WBS Tracker'!B:B,A7,'WBS Tracker'!H:H)</f>
+        <v/>
+      </c>
+      <c r="G7">
+        <f>E7-F7</f>
         <v/>
       </c>
       <c r="H7" s="9">
         <f>IF(B7=0,0,C7/B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Excel Upload</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>COUNTIF('WBS Tracker'!B:B,A8)</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>COUNTIFS('WBS Tracker'!B:B,A8,'WBS Tracker'!J:J,"Completed")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>B8-C8</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>SUMIF('WBS Tracker'!B:B,A8,'WBS Tracker'!G:G)</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>SUMIF('WBS Tracker'!B:B,A8,'WBS Tracker'!H:H)</f>
+        <v/>
+      </c>
+      <c r="G8">
+        <f>E8-F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="9">
+        <f>IF(B8=0,0,C8/B8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B9" s="4">
+        <f>SUM(B5:B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="4">
+        <f>SUM(C5:C8)</f>
+        <v/>
+      </c>
+      <c r="D9" s="4">
+        <f>SUM(D5:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="4">
+        <f>SUM(E5:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="4">
+        <f>SUM(F5:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="4">
+        <f>SUM(G5:G8)</f>
+        <v/>
+      </c>
+      <c r="H9" s="9">
+        <f>IF(B9=0,0,C9/B9)</f>
         <v/>
       </c>
     </row>

</xml_diff>